<commit_message>
feat: tab Top Lojas com ranking top 10 por shopping
Extrai dados de lojas do Snowflake (valor, cupons, clientes, ticket medio).
Nova tab 'Top Lojas' com: filtro por shopping, KPIs, grafico horizontal
top 10, tabela detalhada com ranking. 681 lojas extraidas.
</commit_message>
<xml_diff>
--- a/dados/lojas_nao_cadastradas_snowflake.xlsx
+++ b/dados/lojas_nao_cadastradas_snowflake.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\util\Docker_Airflow\Promocoes_Report\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA41740-36B5-4ECB-BBD5-FBDEEDCBAF1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{865C3160-5C45-401E-B545-A6A865BD3DFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="101">
   <si>
     <t>Shopping ID</t>
   </si>
@@ -43,12 +43,6 @@
     <t>Antonio's Boliche</t>
   </si>
   <si>
-    <t>45954935000145</t>
-  </si>
-  <si>
-    <t>C9 (GIFTCARD)</t>
-  </si>
-  <si>
     <t>63728681000129</t>
   </si>
   <si>
@@ -314,6 +308,21 @@
   </si>
   <si>
     <t>Havanna Café</t>
+  </si>
+  <si>
+    <t>SIM</t>
+  </si>
+  <si>
+    <t>Estava Desabilitado Fidelidade?</t>
+  </si>
+  <si>
+    <t>CNPJ diferente do cadastro no ajfans?</t>
+  </si>
+  <si>
+    <t>NÃO</t>
+  </si>
+  <si>
+    <t>Operação Encerrada</t>
   </si>
 </sst>
 </file>
@@ -654,16 +663,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.21875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.5546875" customWidth="1"/>
     <col min="4" max="4" width="31.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="40.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -676,8 +686,14 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -685,13 +701,19 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -704,8 +726,14 @@
       <c r="D3" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>4</v>
       </c>
@@ -718,8 +746,14 @@
       <c r="D4" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -727,32 +761,44 @@
         <v>5</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
       <c r="B6" s="1" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>88</v>
+        <v>14</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>16</v>
@@ -760,565 +806,711 @@
       <c r="D7" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+        <v>24</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+        <v>94</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>27</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>29</v>
+        <v>88</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C28" s="1" t="s">
+      <c r="D33" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D28" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C29" s="1" t="s">
+      <c r="B34" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D29" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="C34" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+        <v>78</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+        <v>82</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A43" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D43" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D44" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A46" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D46" s="1" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>86</v>
+      <c r="E42" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>